<commit_message>
add new feature flow : Restitusi
</commit_message>
<xml_diff>
--- a/collections/test_script.xlsx
+++ b/collections/test_script.xlsx
@@ -34,7 +34,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -42,12 +42,21 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin"/>
+      <right style="thin"/>
+      <top style="thin"/>
+      <bottom style="thin"/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -413,7 +422,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N44"/>
+  <dimension ref="A1:N48"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -605,8 +614,8 @@
       </c>
       <c r="I4" t="inlineStr">
         <is>
-          <t xml:space="preserve">nomor_transaksi: AKS-20260810-094853-WXZGIP
-ktp: 6621997483706595
+          <t xml:space="preserve">nomor_transaksi: AKS-20260824-101719-SHWAVL
+ktp: 6165647564759970
 </t>
         </is>
       </c>
@@ -629,7 +638,7 @@
       </c>
       <c r="N4" t="inlineStr">
         <is>
-          <t>10/08/2026</t>
+          <t>24/08/2026</t>
         </is>
       </c>
     </row>
@@ -2694,10 +2703,9 @@
       </c>
       <c r="I33" t="inlineStr">
         <is>
-          <t xml:space="preserve">nomor_transaksi: AKS-20260810-093407-SRVUEE
-ktp: 3404387391812951
-nomor_loan: LN-382229
-nomor_loan: LN-035643
+          <t xml:space="preserve">nomor_transaksi: AKS-20260902-161803-BXXUXZ
+ktp: 4604279465860287
+nomor_loan: LN-976237
 </t>
         </is>
       </c>
@@ -2710,7 +2718,7 @@
       </c>
       <c r="K33" t="inlineStr">
         <is>
-          <t>Failed</t>
+          <t>Passed</t>
         </is>
       </c>
       <c r="M33" t="inlineStr">
@@ -2720,7 +2728,7 @@
       </c>
       <c r="N33" t="inlineStr">
         <is>
-          <t>10/08/2026</t>
+          <t>02/09/2026</t>
         </is>
       </c>
     </row>
@@ -2767,9 +2775,9 @@
       </c>
       <c r="I34" t="inlineStr">
         <is>
-          <t xml:space="preserve">nomor_transaksi: AKS-20260814-155028-BXHGYD
-ktp: 7930920405925650
-nomor_loan: LN-383173
+          <t xml:space="preserve">nomor_transaksi: AKS-20260902-145009-WHOOQD
+ktp: 6447939634195919
+nomor_loan: LN-725452
 </t>
         </is>
       </c>
@@ -2792,7 +2800,7 @@
       </c>
       <c r="N34" t="inlineStr">
         <is>
-          <t>14/08/2026</t>
+          <t>02/09/2026</t>
         </is>
       </c>
     </row>
@@ -3190,8 +3198,8 @@
       </c>
       <c r="I40" t="inlineStr">
         <is>
-          <t xml:space="preserve">nomor_transaksi: AKS-20260814-140623-SLFSGB
-ktp: 3168900258421529
+          <t xml:space="preserve">nomor_transaksi: AKS-20260820-155153-PZOEXN
+ktp: 1305984111740260
 </t>
         </is>
       </c>
@@ -3214,7 +3222,7 @@
       </c>
       <c r="N40" t="inlineStr">
         <is>
-          <t>14/08/2026</t>
+          <t>20/08/2026</t>
         </is>
       </c>
     </row>
@@ -3261,8 +3269,8 @@
       </c>
       <c r="I41" t="inlineStr">
         <is>
-          <t xml:space="preserve">nomor_transaksi: AKS-20260814-140832-KVISKL
-ktp: 7360359479212527
+          <t xml:space="preserve">nomor_transaksi: AKS-20260820-155401-TABFQH
+ktp: 0928839527027039
 </t>
         </is>
       </c>
@@ -3285,7 +3293,7 @@
       </c>
       <c r="N41" t="inlineStr">
         <is>
-          <t>14/08/2026</t>
+          <t>20/08/2026</t>
         </is>
       </c>
     </row>
@@ -3332,7 +3340,7 @@
       </c>
       <c r="I42" t="inlineStr">
         <is>
-          <t xml:space="preserve">ktp: 5144664616295173
+          <t xml:space="preserve">ktp: 7046120439275291
 </t>
         </is>
       </c>
@@ -3355,7 +3363,7 @@
       </c>
       <c r="N42" t="inlineStr">
         <is>
-          <t>14/08/2026</t>
+          <t>20/08/2026</t>
         </is>
       </c>
     </row>
@@ -3402,7 +3410,7 @@
       </c>
       <c r="I43" t="inlineStr">
         <is>
-          <t xml:space="preserve">ktp: 8840920497274831
+          <t xml:space="preserve">ktp: 4341979488740436
 </t>
         </is>
       </c>
@@ -3425,7 +3433,7 @@
       </c>
       <c r="N43" t="inlineStr">
         <is>
-          <t>14/08/2026</t>
+          <t>20/08/2026</t>
         </is>
       </c>
     </row>
@@ -3472,8 +3480,8 @@
       </c>
       <c r="I44" t="inlineStr">
         <is>
-          <t xml:space="preserve">nomor_transaksi: AKS-20260814-140846-BXWLLZ
-ktp: 4929626691647152
+          <t xml:space="preserve">nomor_transaksi: AKS-20260820-155416-JNUTVO
+ktp: 8777671845561086
 </t>
         </is>
       </c>
@@ -3496,7 +3504,300 @@
       </c>
       <c r="N44" t="inlineStr">
         <is>
-          <t>14/08/2026</t>
+          <t>20/08/2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="n">
+        <v>42</v>
+      </c>
+      <c r="B45" t="inlineStr">
+        <is>
+          <t>Akseptasi H2H</t>
+        </is>
+      </c>
+      <c r="C45" t="inlineStr">
+        <is>
+          <t>Submit Draft Multi Fasilitas</t>
+        </is>
+      </c>
+      <c r="D45" t="inlineStr">
+        <is>
+          <t>TC-42</t>
+        </is>
+      </c>
+      <c r="E45" t="inlineStr">
+        <is>
+          <t>Multi Fasilitas &gt; 2 Pengajuan (Limit Berjenjang berdasar Outstanding)</t>
+        </is>
+      </c>
+      <c r="F45" t="inlineStr">
+        <is>
+          <t>Negative</t>
+        </is>
+      </c>
+      <c r="G45" t="inlineStr">
+        <is>
+          <t>Simulasi 4 pengajuan berturut-turut pada 1 KTP hingga tahap Inquiry Loan</t>
+        </is>
+      </c>
+      <c r="H45" t="inlineStr">
+        <is>
+          <t>1. Pengajuan 1: Submit (UP 300jt) -&gt; Inquiry (Out: 200jt)
+2. Pengajuan 2: Submit (UP 200jt) -&gt; Inquiry (Out: 200jt)
+3. Pengajuan 3: Submit (UP 100jt) -&gt; Inquiry (Out: 50jt)
+4. Pengajuan 4: Submit (UP 100jt) -&gt; Ditolak (Limit Akumulasi &gt; 500jt)
+5. Validasi DB Tabel Limit Akumulasi</t>
+        </is>
+      </c>
+      <c r="I45" t="inlineStr">
+        <is>
+          <t xml:space="preserve">nomor_transaksi: AKS-20260820-155605-IMZMWW
+ktp: 7908190488617109
+nomor_loan: LN-086688
+nomor_transaksi: AKS-20260820-155605-PYVNNE
+nomor_loan: LN-744052
+nomor_transaksi: AKS-20260820-155606-ZMKZBD
+nomor_loan: LN-009170
+nomor_transaksi: AKS-20260820-155606-LPJWHG
+</t>
+        </is>
+      </c>
+      <c r="J45" t="inlineStr">
+        <is>
+          <t>1. Sistem menolak pengajuan Submit Draft ke-4 karena limit akumulasi (Outstanding lama + UP Baru) &gt; 500 Juta
+2. Data tidak terecord atau termutasi di Database.</t>
+        </is>
+      </c>
+      <c r="K45" t="inlineStr">
+        <is>
+          <t>Passed</t>
+        </is>
+      </c>
+      <c r="N45" t="inlineStr">
+        <is>
+          <t>20/08/2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="n">
+        <v>43</v>
+      </c>
+      <c r="B46" t="inlineStr">
+        <is>
+          <t>Akseptasi H2H</t>
+        </is>
+      </c>
+      <c r="C46" t="inlineStr">
+        <is>
+          <t>Submit Draft Multi Fasilitas</t>
+        </is>
+      </c>
+      <c r="D46" t="inlineStr">
+        <is>
+          <t>TC-43</t>
+        </is>
+      </c>
+      <c r="E46" t="inlineStr">
+        <is>
+          <t>Multi Fasilitas &gt; 2 Pengajuan Sampai Payment (Limit Berjenjang berdasar Outstanding)</t>
+        </is>
+      </c>
+      <c r="F46" t="inlineStr">
+        <is>
+          <t>Negative</t>
+        </is>
+      </c>
+      <c r="G46" t="inlineStr">
+        <is>
+          <t>Simulasi 4 pengajuan berturut-turut pada 1 KTP hingga tahap Payment</t>
+        </is>
+      </c>
+      <c r="H46" t="inlineStr">
+        <is>
+          <t>1. Pengajuan 1: Submit (UP 300jt) -&gt; Inquiry -&gt; Otorisasi -&gt; Payment (Polis Terbit)
+2. Pengajuan 2: Submit (UP 200jt) -&gt; Inquiry -&gt; Otorisasi -&gt; Payment (Polis Terbit)
+3. Pengajuan 3: Submit (UP 100jt) -&gt; Inquiry -&gt; Otorisasi -&gt; Payment (Polis Terbit)
+4. Pengajuan 4: Submit (UP 100jt) -&gt; Ditolak (Limit Akumulasi &gt; 500jt)
+5. Validasi DB Tabel Limit Akumulasi &amp; Pengecekan ACS, FMS</t>
+        </is>
+      </c>
+      <c r="I46" t="inlineStr">
+        <is>
+          <t xml:space="preserve">nomor_transaksi: AKS-20260820-155606-KYTATP
+ktp: 6382463712445182
+nomor_loan: LN-037196
+nomor_transaksi: AKS-20260820-155801-REIUHP
+nomor_loan: LN-577490
+nomor_transaksi: AKS-20260820-155957-DVEWWH
+nomor_loan: LN-674157
+nomor_transaksi: AKS-20260820-160155-MUCZXF
+</t>
+        </is>
+      </c>
+      <c r="J46" t="inlineStr">
+        <is>
+          <t>1. Sistem menolak pengajuan Submit Draft ke-4 karena limit akumulasi (Outstanding lama + UP Baru) &gt; 500 Juta
+2. Data tidak terecord atau termutasi di Database.</t>
+        </is>
+      </c>
+      <c r="K46" t="inlineStr">
+        <is>
+          <t>Passed</t>
+        </is>
+      </c>
+      <c r="N46" t="inlineStr">
+        <is>
+          <t>20/08/2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="n">
+        <v>44</v>
+      </c>
+      <c r="B47" t="inlineStr">
+        <is>
+          <t>Akseptasi H2H</t>
+        </is>
+      </c>
+      <c r="C47" t="inlineStr">
+        <is>
+          <t>Submit Draft Multi Fasilitas</t>
+        </is>
+      </c>
+      <c r="D47" t="inlineStr">
+        <is>
+          <t>TC-44</t>
+        </is>
+      </c>
+      <c r="E47" t="inlineStr">
+        <is>
+          <t>Multi Fasilitas Batal (Reset Kalkulasi)</t>
+        </is>
+      </c>
+      <c r="F47" t="inlineStr">
+        <is>
+          <t>Negative</t>
+        </is>
+      </c>
+      <c r="G47" t="inlineStr">
+        <is>
+          <t>Simulasi pengajuan berturut-turut pada 1 KTP hingga tahap Inquiry Loan, lalu batalkan salah satu, dan ajukan lagi untuk memastikan kalkulasi reset</t>
+        </is>
+      </c>
+      <c r="H47" t="inlineStr">
+        <is>
+          <t>1. Pengajuan 1: Submit (UP 300jt) -&gt; Inquiry (Out: 200jt)
+2. Pengajuan 2: Submit (UP 200jt) -&gt; Inquiry (Out: 200jt)
+3. Pengajuan 3: Submit (UP 100jt) -&gt; Inquiry (Out: 50jt)
+4. Batal Pengajuan 3
+5. Pengajuan 4: Submit (UP 100jt) -&gt; Inquiry (Out: 100jt)
+6. Pengajuan 5: Submit (UP 50jt) -&gt; Ditolak (Limit Akumulasi &gt; 500jt)</t>
+        </is>
+      </c>
+      <c r="I47" t="inlineStr">
+        <is>
+          <t xml:space="preserve">nomor_transaksi: AKS-20260820-160155-CQTSOQ
+ktp: 9777963197043459
+nomor_loan: LN-330350
+nomor_transaksi: AKS-20260820-160155-KRYSMR
+nomor_loan: LN-376753
+nomor_transaksi: AKS-20260820-160156-VVXJZW
+nomor_loan: LN-300776
+nomor_transaksi: AKS-20260820-160156-QYCXYK
+nomor_loan: LN-379387
+nomor_transaksi: AKS-20260820-160156-UFWMIK
+</t>
+        </is>
+      </c>
+      <c r="J47" t="inlineStr">
+        <is>
+          <t>1. Sistem menerima pengajuan setelah ada pembatalan, dan menolak pengajuan terakhir karena limit akumulasi (Outstanding lama + UP Baru) &gt; 500 Juta
+2. Data tidak terecord atau termutasi di Database.</t>
+        </is>
+      </c>
+      <c r="K47" t="inlineStr">
+        <is>
+          <t>Passed</t>
+        </is>
+      </c>
+      <c r="N47" t="inlineStr">
+        <is>
+          <t>20/08/2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="n">
+        <v>45</v>
+      </c>
+      <c r="B48" t="inlineStr">
+        <is>
+          <t>Akseptasi H2H</t>
+        </is>
+      </c>
+      <c r="C48" t="inlineStr">
+        <is>
+          <t>Submit Draft Multi Fasilitas</t>
+        </is>
+      </c>
+      <c r="D48" t="inlineStr">
+        <is>
+          <t>TC-45</t>
+        </is>
+      </c>
+      <c r="E48" t="inlineStr">
+        <is>
+          <t>Validasi Response Nilai Akumulasi Limit Multi Fasilitas</t>
+        </is>
+      </c>
+      <c r="F48" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="G48" t="inlineStr">
+        <is>
+          <t>KTP belum memiliki fasilitas aktif. Hit menggunakan API Automation.</t>
+        </is>
+      </c>
+      <c r="H48" t="inlineStr">
+        <is>
+          <t>1. Pengajuan 1: Submit Draft (UP 300 Juta) -&gt; Inquiry Loan (Outstanding 100 Juta)
+2. Pengajuan 2: Submit Draft (UP 100 Juta)
+3. Validasi field nilai_akumulasi pada Response API Pengajuan 2
+4. Menampilkan Tabel Validasi Response Nilai Akumulasi</t>
+        </is>
+      </c>
+      <c r="I48" t="inlineStr">
+        <is>
+          <t xml:space="preserve">nomor_transaksi: AKS-20260820-160156-MWWBUF
+ktp: 9207441215116180
+nomor_loan: LN-875740
+nomor_transaksi: AKS-20260820-160157-THXRWK
+nomor_loan: LN-479646
+</t>
+        </is>
+      </c>
+      <c r="J48" t="inlineStr">
+        <is>
+          <t>1. Sistem memproses pengajuan 2 dengan sukses.
+2. Field nilai_akumulasi pada response sesuai dengan total akumulasi (Outstanding lama + UP Baru).
+3. Tabel validasi menampilkan hasil perbandingan yang sesuai.
+4. Data tersimpan dan termutasi dengan benar di Database PostgreSQL.</t>
+        </is>
+      </c>
+      <c r="K48" t="inlineStr">
+        <is>
+          <t>Passed</t>
+        </is>
+      </c>
+      <c r="N48" t="inlineStr">
+        <is>
+          <t>20/08/2026</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
penambahan fitur hold dan penyesuaian nilai restitusi
</commit_message>
<xml_diff>
--- a/collections/test_script.xlsx
+++ b/collections/test_script.xlsx
@@ -450,7 +450,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N60"/>
+  <dimension ref="A1:N69"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="4" customWidth="1" min="1" max="1"/>
@@ -2790,9 +2790,9 @@
       </c>
       <c r="I34" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">nomor_transaksi: AKS-20260929-110409-HMUNZL
-ktp: 8347158403760416
-nomor_loan: LN-252707
+          <t xml:space="preserve">nomor_transaksi: AKS-20261007-082831-THKAYE
+ktp: 2781845484047191
+nomor_loan: LN-249375
 </t>
         </is>
       </c>
@@ -2816,7 +2816,7 @@
       </c>
       <c r="N34" s="1" t="inlineStr">
         <is>
-          <t>29/09/2026</t>
+          <t>07/10/2026</t>
         </is>
       </c>
     </row>
@@ -4125,8 +4125,8 @@
       </c>
       <c r="I52" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">nomor_transaksi: AKS-20260925-153909-NBFDNU
-ktp: 0640951844203473
+          <t xml:space="preserve">nomor_transaksi: AKS-20261005-100916-MPRAIR
+ktp: 0984266348951664
 </t>
         </is>
       </c>
@@ -4173,7 +4173,7 @@
       </c>
       <c r="N52" s="1" t="inlineStr">
         <is>
-          <t>25/09/2026</t>
+          <t>05/10/2026</t>
         </is>
       </c>
     </row>
@@ -4900,6 +4900,640 @@
         </is>
       </c>
     </row>
+    <row r="61">
+      <c r="A61" s="1" t="n">
+        <v>58</v>
+      </c>
+      <c r="B61" s="1" t="inlineStr">
+        <is>
+          <t>Akseptasi</t>
+        </is>
+      </c>
+      <c r="C61" s="1" t="inlineStr">
+        <is>
+          <t>API - Submit Draft Akseptasi</t>
+        </is>
+      </c>
+      <c r="D61" s="1" t="inlineStr">
+        <is>
+          <t>TC-58</t>
+        </is>
+      </c>
+      <c r="E61" s="1" t="inlineStr">
+        <is>
+          <t>Penolakan akseptasi menggunakan data debitur berstatus blacklist di Askrindo</t>
+        </is>
+      </c>
+      <c r="F61" s="1" t="inlineStr">
+        <is>
+          <t>Negative</t>
+        </is>
+      </c>
+      <c r="G61" s="1" t="inlineStr">
+        <is>
+          <t>Mengambil data NIK debitur blacklist dari DB ACS</t>
+        </is>
+      </c>
+      <c r="H61" s="1" t="inlineStr">
+        <is>
+          <t>1. Hit API Submit Draft Akseptasi menggunakan NIK debitur berstatus blacklist.
+2. Memvalidasi respon API terhadap penolakan.</t>
+        </is>
+      </c>
+      <c r="I61" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">nomor_transaksi: AKS-20261007-133944-PKYKQX
+ktp: 0950074704632002
+</t>
+        </is>
+      </c>
+      <c r="J61" s="1" t="inlineStr">
+        <is>
+          <t>1. API menolak pengajuan akseptasi.
+2. Message: Akseptasi Ditolak, Debitur dalam Status Blacklist Askrindo
+3. Data tidak terecord atau termutasi di Database.</t>
+        </is>
+      </c>
+      <c r="K61" s="4" t="inlineStr">
+        <is>
+          <t>Passed</t>
+        </is>
+      </c>
+      <c r="L61" s="1" t="inlineStr"/>
+      <c r="M61" s="1" t="inlineStr">
+        <is>
+          <t>Fathur</t>
+        </is>
+      </c>
+      <c r="N61" s="1" t="inlineStr">
+        <is>
+          <t>07/10/2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" s="1" t="n">
+        <v>59</v>
+      </c>
+      <c r="B62" s="1" t="inlineStr">
+        <is>
+          <t>Restitusi</t>
+        </is>
+      </c>
+      <c r="C62" s="1" t="inlineStr">
+        <is>
+          <t>API - Restitusi Confirmation</t>
+        </is>
+      </c>
+      <c r="D62" s="1" t="inlineStr">
+        <is>
+          <t>TC-59</t>
+        </is>
+      </c>
+      <c r="E62" s="1" t="inlineStr">
+        <is>
+          <t>Persetujuan restitusi berdasarkan nilai terkecil dari input konfirmasi (Pengajuan Awal &lt; Kalkulasi)</t>
+        </is>
+      </c>
+      <c r="F62" s="1" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="G62" s="1" t="inlineStr">
+        <is>
+          <t>Polis Terbit</t>
+        </is>
+      </c>
+      <c r="H62" s="1" t="inlineStr">
+        <is>
+          <t>1. Hit API Submit Restitusi dengan nilai pengajuan lebih kecil dari kalkulasi Askrindo.
+2. Hit API Konfirmasi Restitusi dengan nilai konfirmasi lebih kecil dari nilai pengajuan.
+3. Melakukan Validasi DB pada setiap langkah.</t>
+        </is>
+      </c>
+      <c r="I62" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">nomor_transaksi: AKS-20261007-091506-FMSYRM
+ktp: 0598891781029431
+</t>
+        </is>
+      </c>
+      <c r="J62" s="1" t="inlineStr">
+        <is>
+          <t>1. Sistem mencatat dan menyetujui nilai restitusi berdasarkan input konfirmasi (nilai terkecil).
+2. Data ter-update benar di DB.
+3. Data tersimpan dan termutasi dengan benar di Database PostgreSQL.</t>
+        </is>
+      </c>
+      <c r="K62" s="4" t="inlineStr">
+        <is>
+          <t>Passed</t>
+        </is>
+      </c>
+      <c r="L62" s="1" t="inlineStr"/>
+      <c r="M62" s="1" t="inlineStr">
+        <is>
+          <t>Fathur</t>
+        </is>
+      </c>
+      <c r="N62" s="1" t="inlineStr">
+        <is>
+          <t>07/10/2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" s="1" t="n">
+        <v>60</v>
+      </c>
+      <c r="B63" s="1" t="inlineStr">
+        <is>
+          <t>Restitusi</t>
+        </is>
+      </c>
+      <c r="C63" s="1" t="inlineStr">
+        <is>
+          <t>API - Restitusi Dispute</t>
+        </is>
+      </c>
+      <c r="D63" s="1" t="inlineStr">
+        <is>
+          <t>TC-60</t>
+        </is>
+      </c>
+      <c r="E63" s="1" t="inlineStr">
+        <is>
+          <t>Persetujuan restitusi setelah proses sanggahan yang memenuhi kalkulasi Askrindo</t>
+        </is>
+      </c>
+      <c r="F63" s="1" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="G63" s="1" t="inlineStr">
+        <is>
+          <t>Polis Terbit</t>
+        </is>
+      </c>
+      <c r="H63" s="1" t="inlineStr">
+        <is>
+          <t>1. Hit API Submit Restitusi dengan nilai pengajuan lebih besar dari kalkulasi (Sanggahan).
+2. Hit API Dispute/Sanggahan dengan menginput nilai &lt;= kalkulasi Askrindo.
+3. Melakukan Validasi DB.</t>
+        </is>
+      </c>
+      <c r="I63" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">nomor_transaksi: AKS-20261007-091507-PFQJMK
+ktp: 0598891781029431
+</t>
+        </is>
+      </c>
+      <c r="J63" s="1" t="inlineStr">
+        <is>
+          <t>1. Sanggahan disetujui otomatis setelah nilai memenuhi batas.
+2. Data tersimpan dan termutasi dengan benar di Database PostgreSQL.</t>
+        </is>
+      </c>
+      <c r="K63" s="4" t="inlineStr">
+        <is>
+          <t>Failed</t>
+        </is>
+      </c>
+      <c r="L63" s="1" t="inlineStr"/>
+      <c r="M63" s="1" t="inlineStr">
+        <is>
+          <t>Fathur</t>
+        </is>
+      </c>
+      <c r="N63" s="1" t="inlineStr">
+        <is>
+          <t>07/10/2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" s="1" t="n">
+        <v>61</v>
+      </c>
+      <c r="B64" s="1" t="inlineStr">
+        <is>
+          <t>Restitusi</t>
+        </is>
+      </c>
+      <c r="C64" s="1" t="inlineStr">
+        <is>
+          <t>API - Restitusi Dispute</t>
+        </is>
+      </c>
+      <c r="D64" s="1" t="inlineStr">
+        <is>
+          <t>TC-61</t>
+        </is>
+      </c>
+      <c r="E64" s="1" t="inlineStr">
+        <is>
+          <t>Penolakan sanggahan restitusi ilegal dengan nilai lebih besar dari pengajuan awal</t>
+        </is>
+      </c>
+      <c r="F64" s="1" t="inlineStr">
+        <is>
+          <t>Negative</t>
+        </is>
+      </c>
+      <c r="G64" s="1" t="inlineStr">
+        <is>
+          <t>Polis Terbit</t>
+        </is>
+      </c>
+      <c r="H64" s="1" t="inlineStr">
+        <is>
+          <t>1. Hit API Submit Restitusi dengan nilai pengajuan awal di bawah batas kalkulasi.
+2. Hit API Sanggahan dengan memasukkan nilai yang lebih besar dari nilai pengajuan awal.
+3. Memvalidasi respon API penolakan.</t>
+        </is>
+      </c>
+      <c r="I64" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">nomor_transaksi: AKS-20261007-091509-TIZTVB
+ktp: 0598891781029431
+</t>
+        </is>
+      </c>
+      <c r="J64" s="1" t="inlineStr">
+        <is>
+          <t>1. API menolak proses sanggahan (HTTP 400).
+2. Data tersimpan dan termutasi dengan benar di Database PostgreSQL.</t>
+        </is>
+      </c>
+      <c r="K64" s="4" t="inlineStr">
+        <is>
+          <t>Failed</t>
+        </is>
+      </c>
+      <c r="L64" s="1" t="inlineStr"/>
+      <c r="M64" s="1" t="inlineStr">
+        <is>
+          <t>Fathur</t>
+        </is>
+      </c>
+      <c r="N64" s="1" t="inlineStr">
+        <is>
+          <t>07/10/2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" s="1" t="n">
+        <v>62</v>
+      </c>
+      <c r="B65" s="1" t="inlineStr">
+        <is>
+          <t>Restitusi</t>
+        </is>
+      </c>
+      <c r="C65" s="1" t="inlineStr">
+        <is>
+          <t>API - Restitusi</t>
+        </is>
+      </c>
+      <c r="D65" s="1" t="inlineStr">
+        <is>
+          <t>TC-62</t>
+        </is>
+      </c>
+      <c r="E65" s="1" t="inlineStr">
+        <is>
+          <t>Pengajuan restitusi berstatus hold untuk premi belum lunas dan dilanjutkan otomatis hingga persetujuan</t>
+        </is>
+      </c>
+      <c r="F65" s="1" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="G65" s="1" t="inlineStr">
+        <is>
+          <t>Draft Akseptasi sampai Otorisasi tanpa pelunasan premi</t>
+        </is>
+      </c>
+      <c r="H65" s="1" t="inlineStr">
+        <is>
+          <t>1. Hit API Submit Restitusi saat premi belum lunas.
+2. Validasi status akseptasi di DB menjadi 12 (Hold).
+3. Melakukan patching lunas pada premi di DB ACS.
+4. Menunggu scheduler memperbarui status akseptasi menjadi 13.
+5. Lanjutkan konfirmasi hingga selesai.</t>
+        </is>
+      </c>
+      <c r="I65" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">nomor_transaksi: AKS-20261007-091510-BCKBTI
+ktp: 0598891781029431
+</t>
+        </is>
+      </c>
+      <c r="J65" s="1" t="inlineStr">
+        <is>
+          <t>1. API merespon pengajuan ditahan (Hold).
+2. Status otomatis berubah ke 13 setelah lunas.
+3. Alur konfirmasi berhasil dilakukan.
+4. Data tersimpan dan termutasi dengan benar di Database PostgreSQL.</t>
+        </is>
+      </c>
+      <c r="K65" s="4" t="inlineStr">
+        <is>
+          <t>Failed</t>
+        </is>
+      </c>
+      <c r="L65" s="1" t="inlineStr"/>
+      <c r="M65" s="1" t="inlineStr">
+        <is>
+          <t>Fathur</t>
+        </is>
+      </c>
+      <c r="N65" s="1" t="inlineStr">
+        <is>
+          <t>07/10/2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" s="1" t="n">
+        <v>63</v>
+      </c>
+      <c r="B66" s="1" t="inlineStr">
+        <is>
+          <t>Akseptasi H2H</t>
+        </is>
+      </c>
+      <c r="C66" s="1" t="inlineStr">
+        <is>
+          <t>A8 - Restitusi</t>
+        </is>
+      </c>
+      <c r="D66" s="1" t="inlineStr">
+        <is>
+          <t>TC-63</t>
+        </is>
+      </c>
+      <c r="E66" s="1" t="inlineStr">
+        <is>
+          <t>Submit Restitusi dengan Nomor Loan yang sudah memiliki pengajuan restitusi aktif (Double Submit)</t>
+        </is>
+      </c>
+      <c r="F66" s="1" t="inlineStr">
+        <is>
+          <t>Negative</t>
+        </is>
+      </c>
+      <c r="G66" s="1" t="inlineStr">
+        <is>
+          <t>Terdapat Polis Terbit dan sudah ada pengajuan restitusi yang belum berstatus batal/selesai</t>
+        </is>
+      </c>
+      <c r="H66" s="1" t="inlineStr">
+        <is>
+          <t>1. Hit API Submit Restitusi Pertama (Sukses)
+2. Hit API Submit Restitusi Kedua menggunakan nomor loan yang sama</t>
+        </is>
+      </c>
+      <c r="I66" s="1" t="n"/>
+      <c r="J66" s="1" t="inlineStr">
+        <is>
+          <t>1. Sistem menolak dengan HTTP 422.
+2. Muncul pesan validasi bahwa nomor loan sedang dalam proses restitusi.</t>
+        </is>
+      </c>
+      <c r="K66" s="4" t="n"/>
+      <c r="L66" s="1" t="n"/>
+      <c r="M66" s="1" t="n"/>
+      <c r="N66" s="1" t="n"/>
+    </row>
+    <row r="67">
+      <c r="A67" s="1" t="n">
+        <v>64</v>
+      </c>
+      <c r="B67" s="1" t="inlineStr">
+        <is>
+          <t>Restitusi</t>
+        </is>
+      </c>
+      <c r="C67" s="1" t="inlineStr">
+        <is>
+          <t>API - Restitusi Confirmation</t>
+        </is>
+      </c>
+      <c r="D67" s="1" t="inlineStr">
+        <is>
+          <t>TC-64</t>
+        </is>
+      </c>
+      <c r="E67" s="1" t="inlineStr">
+        <is>
+          <t>Penolakan konfirmasi restitusi ilegal dengan nilai lebih besar dari pengajuan awal</t>
+        </is>
+      </c>
+      <c r="F67" s="1" t="inlineStr">
+        <is>
+          <t>Negative</t>
+        </is>
+      </c>
+      <c r="G67" s="1" t="inlineStr">
+        <is>
+          <t>Polis Terbit</t>
+        </is>
+      </c>
+      <c r="H67" s="1" t="inlineStr">
+        <is>
+          <t>1. Hit API Submit Restitusi dengan nilai pengajuan awal di bawah batas kalkulasi.
+2. Hit API Konfirmasi (DISETUJUI) dengan memasukkan nilai yang lebih besar dari nilai pengajuan awal.
+3. Memvalidasi respon API penolakan.</t>
+        </is>
+      </c>
+      <c r="I67" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">nomor_transaksi: AKS-20261007-091511-DRWEHX
+ktp: 0598891781029431
+</t>
+        </is>
+      </c>
+      <c r="J67" s="1" t="inlineStr">
+        <is>
+          <t>1. API menolak proses konfirmasi (HTTP 400).
+2. Data tersimpan dan termutasi dengan benar di Database PostgreSQL.</t>
+        </is>
+      </c>
+      <c r="K67" s="4" t="inlineStr">
+        <is>
+          <t>Failed</t>
+        </is>
+      </c>
+      <c r="L67" s="1" t="inlineStr"/>
+      <c r="M67" s="1" t="inlineStr">
+        <is>
+          <t>Fathur</t>
+        </is>
+      </c>
+      <c r="N67" s="1" t="inlineStr">
+        <is>
+          <t>07/10/2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" s="1" t="n">
+        <v>65</v>
+      </c>
+      <c r="B68" s="1" t="inlineStr">
+        <is>
+          <t>Akseptasi</t>
+        </is>
+      </c>
+      <c r="C68" s="1" t="inlineStr">
+        <is>
+          <t>API - Notifikasi Pembayaran</t>
+        </is>
+      </c>
+      <c r="D68" s="1" t="inlineStr">
+        <is>
+          <t>TC-65</t>
+        </is>
+      </c>
+      <c r="E68" s="1" t="inlineStr">
+        <is>
+          <t>E2E Akseptasi murni tanpa dilunasi di sistem ACS</t>
+        </is>
+      </c>
+      <c r="F68" s="1" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="G68" s="1" t="inlineStr">
+        <is>
+          <t>Polis Terbit di Backend</t>
+        </is>
+      </c>
+      <c r="H68" s="1" t="inlineStr">
+        <is>
+          <t>1. Hit API Submit Draft Akseptasi
+2. Hit API Inquiry Loan
+3. Hit API Otorisasi Penyelia
+4. Hit API Payment
+5. Melakukan DB Validation</t>
+        </is>
+      </c>
+      <c r="I68" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">nomor_transaksi: AKS-20261007-095307-IYGKCR
+ktp: 3682091275928871
+nomor_loan: LN-130619
+</t>
+        </is>
+      </c>
+      <c r="J68" s="1" t="inlineStr">
+        <is>
+          <t>1. API berhasil memproses seluruh request (HTTP 200 OK).
+2. Status akseptasi menjadi 9 di PostgreSQL tanpa dimutasi lunas di ACS.
+3. Data tersimpan dan termutasi dengan benar di Database PostgreSQL.</t>
+        </is>
+      </c>
+      <c r="K68" s="4" t="inlineStr">
+        <is>
+          <t>Passed</t>
+        </is>
+      </c>
+      <c r="L68" s="1" t="inlineStr"/>
+      <c r="M68" s="1" t="inlineStr">
+        <is>
+          <t>Fathur</t>
+        </is>
+      </c>
+      <c r="N68" s="1" t="inlineStr">
+        <is>
+          <t>07/10/2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" s="1" t="n">
+        <v>66</v>
+      </c>
+      <c r="B69" s="1" t="inlineStr">
+        <is>
+          <t>Akseptasi</t>
+        </is>
+      </c>
+      <c r="C69" s="1" t="inlineStr">
+        <is>
+          <t>API - Submit Draft Akseptasi</t>
+        </is>
+      </c>
+      <c r="D69" s="1" t="inlineStr">
+        <is>
+          <t>TC-66</t>
+        </is>
+      </c>
+      <c r="E69" s="1" t="inlineStr">
+        <is>
+          <t>E2E Akseptasi menggunakan data debitur yang telah diputihkan (IS_BLACKLIST = 0)</t>
+        </is>
+      </c>
+      <c r="F69" s="1" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="G69" s="1" t="inlineStr">
+        <is>
+          <t>Pemutihan status blacklist debitur di DB ACS (Patch ke 0)</t>
+        </is>
+      </c>
+      <c r="H69" s="1" t="inlineStr">
+        <is>
+          <t>1. Set IS_BLACKLIST = 0 di ACS
+2. Hit API Submit Draft Akseptasi
+3. Hit API Inquiry Loan
+4. Hit API Otorisasi Penyelia
+5. Hit API Payment
+6. Melakukan DB Validation</t>
+        </is>
+      </c>
+      <c r="I69" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">nomor_transaksi: AKS-20261007-094039-BRGNKJ
+ktp: 0950074506770374
+nomor_loan: LN-374331
+</t>
+        </is>
+      </c>
+      <c r="J69" s="1" t="inlineStr">
+        <is>
+          <t>1. API berhasil memproses seluruh request (HTTP 200 OK).
+2. Debitur tidak lagi diblokir dan proses akseptasi berjalan lancar hingga status 9.
+3. Data tersimpan dan termutasi dengan benar di Database PostgreSQL.</t>
+        </is>
+      </c>
+      <c r="K69" s="4" t="inlineStr">
+        <is>
+          <t>Passed</t>
+        </is>
+      </c>
+      <c r="L69" s="1" t="inlineStr"/>
+      <c r="M69" s="1" t="inlineStr">
+        <is>
+          <t>Fathur</t>
+        </is>
+      </c>
+      <c r="N69" s="1" t="inlineStr">
+        <is>
+          <t>07/10/2026</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <mergeCells count="1">
     <mergeCell ref="A1:N2"/>

</xml_diff>